<commit_message>
Still working on the JSON file
</commit_message>
<xml_diff>
--- a/spreadsheet.xlsx
+++ b/spreadsheet.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="305">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="304">
   <si>
     <t>product_id</t>
   </si>
@@ -46,45 +46,45 @@
     <t>13993095</t>
   </si>
   <si>
+    <t>13993244</t>
+  </si>
+  <si>
     <t>13992951</t>
   </si>
   <si>
-    <t>13993244</t>
-  </si>
-  <si>
     <t>13993093</t>
   </si>
   <si>
     <t>12547939</t>
   </si>
   <si>
+    <t>13991952</t>
+  </si>
+  <si>
     <t>12755140</t>
   </si>
   <si>
-    <t>13991952</t>
-  </si>
-  <si>
     <t>12534144</t>
   </si>
   <si>
     <t>12547936</t>
   </si>
   <si>
+    <t>13993381</t>
+  </si>
+  <si>
     <t>13538152</t>
   </si>
   <si>
-    <t>13993381</t>
-  </si>
-  <si>
     <t>13993243</t>
   </si>
   <si>
+    <t>13564531</t>
+  </si>
+  <si>
     <t>13570649</t>
   </si>
   <si>
-    <t>13564531</t>
-  </si>
-  <si>
     <t>13994392</t>
   </si>
   <si>
@@ -100,24 +100,24 @@
     <t>13991987</t>
   </si>
   <si>
+    <t>13567220</t>
+  </si>
+  <si>
+    <t>13994348</t>
+  </si>
+  <si>
+    <t>13992308</t>
+  </si>
+  <si>
     <t>13993303</t>
   </si>
   <si>
-    <t>13992308</t>
-  </si>
-  <si>
-    <t>13994348</t>
+    <t>13992942</t>
   </si>
   <si>
     <t>12534152</t>
   </si>
   <si>
-    <t>13567220</t>
-  </si>
-  <si>
-    <t>13992942</t>
-  </si>
-  <si>
     <t>13994192</t>
   </si>
   <si>
@@ -127,16 +127,34 @@
     <t>12755141</t>
   </si>
   <si>
+    <t>13991991</t>
+  </si>
+  <si>
+    <t>13186208</t>
+  </si>
+  <si>
     <t>13340189</t>
   </si>
   <si>
-    <t>13991991</t>
+    <t>13994264</t>
+  </si>
+  <si>
+    <t>13994393</t>
+  </si>
+  <si>
+    <t>13994235</t>
   </si>
   <si>
     <t>13992135</t>
   </si>
   <si>
-    <t>13186208</t>
+    <t>12481774</t>
+  </si>
+  <si>
+    <t>13993126</t>
+  </si>
+  <si>
+    <t>13994236</t>
   </si>
   <si>
     <t>12474762</t>
@@ -145,39 +163,21 @@
     <t>13340176</t>
   </si>
   <si>
-    <t>13994393</t>
-  </si>
-  <si>
-    <t>13994264</t>
-  </si>
-  <si>
-    <t>13994235</t>
-  </si>
-  <si>
-    <t>12481774</t>
-  </si>
-  <si>
-    <t>13993126</t>
-  </si>
-  <si>
-    <t>13994236</t>
+    <t>13992383</t>
+  </si>
+  <si>
+    <t>13994350</t>
   </si>
   <si>
     <t>13994245</t>
   </si>
   <si>
-    <t>13992383</t>
-  </si>
-  <si>
-    <t>13994350</t>
+    <t>13993089</t>
   </si>
   <si>
     <t>13994352</t>
   </si>
   <si>
-    <t>13993089</t>
-  </si>
-  <si>
     <t>13994360</t>
   </si>
   <si>
@@ -190,22 +190,22 @@
     <t>12481790</t>
   </si>
   <si>
+    <t>13992139</t>
+  </si>
+  <si>
     <t>13340173</t>
   </si>
   <si>
-    <t>13992139</t>
-  </si>
-  <si>
     <t>12547997</t>
   </si>
   <si>
+    <t>13992941</t>
+  </si>
+  <si>
     <t>13340177</t>
   </si>
   <si>
-    <t>13992941</t>
-  </si>
-  <si>
-    <t>13992144</t>
+    <t>13918863</t>
   </si>
   <si>
     <t>13341612</t>
@@ -226,45 +226,45 @@
     <t>Celular Samsung Galaxy S25 FE 5G 128GB 8 GB</t>
   </si>
   <si>
+    <t>Celular Samsung Galaxy A07 4G 128GB 4 GB</t>
+  </si>
+  <si>
     <t>Celular Samsung Galaxy A17 5G 256GB 8 GB</t>
   </si>
   <si>
-    <t>Celular Samsung Galaxy A07 4G 128GB 4 GB</t>
-  </si>
-  <si>
     <t>Celular Samsung Galaxy S25 FE 5G 256GB 8 GB</t>
   </si>
   <si>
     <t>Celular Samsung Galaxy S24 Ultra 5G 256GB 12 GB</t>
   </si>
   <si>
+    <t>iPhone 16e 128GB 8 GB</t>
+  </si>
+  <si>
     <t>iPhone 16 128GB</t>
   </si>
   <si>
-    <t>iPhone 16e 128GB 8 GB</t>
-  </si>
-  <si>
     <t>iPhone 15 128GB 6GB</t>
   </si>
   <si>
     <t>Celular Samsung Galaxy S24 5G 256GB 8 GB</t>
   </si>
   <si>
+    <t>Celular Motorola Moto G G86 5G 256GB 8 GB</t>
+  </si>
+  <si>
     <t>Celular Samsung Galaxy S25 Plus 5G 256GB 12 GB</t>
   </si>
   <si>
-    <t>Celular Motorola Moto G G86 5G 256GB 8 GB</t>
-  </si>
-  <si>
     <t>Celular Samsung Galaxy A07 4G 256GB 8 GB</t>
   </si>
   <si>
+    <t>Celular Samsung Galaxy S25 Ultra 5G 256GB 12 GB</t>
+  </si>
+  <si>
     <t>Celular Samsung Galaxy S25 5G 256GB 12 GB</t>
   </si>
   <si>
-    <t>Celular Samsung Galaxy S25 Ultra 5G 256GB 12 GB</t>
-  </si>
-  <si>
     <t>Celular Samsung A57 256GB 8 GB</t>
   </si>
   <si>
@@ -280,24 +280,24 @@
     <t>Celular Samsung Galaxy A36 5G SM-A366E 128GB 6 GB</t>
   </si>
   <si>
+    <t>Celular Samsung Galaxy S25 Ultra 5G SM-S938B 512GB 12 GB</t>
+  </si>
+  <si>
+    <t>Celular Xiaomi Pocophone Poco X8 Pro 256GB 8 GB</t>
+  </si>
+  <si>
+    <t>Celular Motorola Moto Edge 60 Pro 5G 256GB 12 GB</t>
+  </si>
+  <si>
     <t>Celular Xiaomi Redmi 15 256GB 8 GB</t>
   </si>
   <si>
-    <t>Celular Motorola Moto Edge 60 Pro 5G 256GB 12 GB</t>
-  </si>
-  <si>
-    <t>Celular Xiaomi Pocophone Poco X8 Pro 256GB 8 GB</t>
+    <t>iPhone 17 Pro 256GB</t>
   </si>
   <si>
     <t>iPhone 15 Pro Max 8 GB 256GB</t>
   </si>
   <si>
-    <t>Celular Samsung Galaxy S25 Ultra 5G SM-S938B 512GB 12 GB</t>
-  </si>
-  <si>
-    <t>iPhone 17 Pro 256GB</t>
-  </si>
-  <si>
     <t>Celular Samsung Galaxy S26 Ultra 5G 256GB 12 GB</t>
   </si>
   <si>
@@ -307,16 +307,34 @@
     <t>iPhone 16 256GB</t>
   </si>
   <si>
+    <t>Celular Samsung Galaxy A26 5G SM-A266M 256GB 8 GB</t>
+  </si>
+  <si>
+    <t>Celular Samsung Galaxy S24 FE 5G 256GB 8 GB</t>
+  </si>
+  <si>
     <t>Celular Samsung Galaxy A25 5G 256GB 8 GB</t>
   </si>
   <si>
-    <t>Celular Samsung Galaxy A26 5G SM-A266M 256GB 8 GB</t>
+    <t>Celular Motorola Edge 70 Fusion 5G 256GB 8 GB</t>
+  </si>
+  <si>
+    <t>Celular Samsung A57 128GB 8 GB</t>
+  </si>
+  <si>
+    <t>Celular Samsung Galaxy A17 4G 128GB 4 GB</t>
   </si>
   <si>
     <t>Celular Motorola Moto Edge 60 Fusion 5G 256GB 8 GB</t>
   </si>
   <si>
-    <t>Celular Samsung Galaxy S24 FE 5G 256GB 8 GB</t>
+    <t>iPhone 14 Plus 256GB 6GB</t>
+  </si>
+  <si>
+    <t>Celular Xiaomi Poco C85 256GB 8 GB</t>
+  </si>
+  <si>
+    <t>Celular Samsung Galaxy A17 4G 256GB 8 GB</t>
   </si>
   <si>
     <t>iPhone 13 4 GB 256GB</t>
@@ -325,39 +343,21 @@
     <t>Celular Motorola Moto G35 5G 128GB 12 GB</t>
   </si>
   <si>
-    <t>Celular Samsung A57 128GB 8 GB</t>
-  </si>
-  <si>
-    <t>Celular Motorola Edge 70 Fusion 5G 256GB 8 GB</t>
-  </si>
-  <si>
-    <t>Celular Samsung Galaxy A17 4G 128GB 4 GB</t>
-  </si>
-  <si>
-    <t>iPhone 14 Plus 256GB 6GB</t>
-  </si>
-  <si>
-    <t>Celular Xiaomi Poco C85 256GB 8 GB</t>
-  </si>
-  <si>
-    <t>Celular Samsung Galaxy A17 4G 256GB 8 GB</t>
+    <t>Celular Motorola Moto G G56 5G 256GB 8 GB</t>
+  </si>
+  <si>
+    <t>Celular Xiaomi Pocophone Poco X8 Pro 512GB 12 GB</t>
   </si>
   <si>
     <t>Celular Apple iPhone 17e 5G 256GB</t>
   </si>
   <si>
-    <t>Celular Motorola Moto G G56 5G 256GB 8 GB</t>
-  </si>
-  <si>
-    <t>Celular Xiaomi Pocophone Poco X8 Pro 512GB 12 GB</t>
+    <t>Celular Motorola Moto G G06 128GB 4 GB</t>
   </si>
   <si>
     <t>Celular Xiaomi Pocophone Poco X8 Pro Max 512GB 12 GB</t>
   </si>
   <si>
-    <t>Celular Motorola Moto G G06 128GB 4 GB</t>
-  </si>
-  <si>
     <t>Celular Xiaomi Redmi Note 15 Pro 5G 256GB 8 GB</t>
   </si>
   <si>
@@ -370,22 +370,22 @@
     <t>Celular Apple iPhone 14 Pro 256GB 6 GB</t>
   </si>
   <si>
+    <t>Celular Motorola Edge 60 5G XT2505-4 512GB 12 GB</t>
+  </si>
+  <si>
     <t>Celular Motorola Moto G35 5G 256GB 12 GB</t>
   </si>
   <si>
-    <t>Celular Motorola Edge 60 5G XT2505-4 512GB 12 GB</t>
-  </si>
-  <si>
     <t>Celular Samsung Galaxy A05s 128GB 6 GB</t>
   </si>
   <si>
+    <t>iPhone 17 Pro Max 512GB</t>
+  </si>
+  <si>
     <t>Celular Motorola Moto G75 5G XT2437-2 256GB 16 GB</t>
   </si>
   <si>
-    <t>iPhone 17 Pro Max 512GB</t>
-  </si>
-  <si>
-    <t>Celular Motorola Moto Edge 60 Pro 5G 512GB 12 GB</t>
+    <t>Celular Xiaomi Redmi Note 14 Pro 5G 256GB 8 GB</t>
   </si>
   <si>
     <t>Celular Xiaomi Poco X7 Pro 5G 256GB 8 GB</t>
@@ -406,45 +406,45 @@
     <t>/celular/celular-samsung-galaxy-s25-fe-5g-128gb-8-gb?_lc=11</t>
   </si>
   <si>
+    <t>/celular/celular-samsung-galaxy-a07-4g-128gb-4-gb?_lc=11</t>
+  </si>
+  <si>
     <t>/celular/celular-samsung-galaxy-a17-256gb-8-gb?_lc=11</t>
   </si>
   <si>
-    <t>/celular/celular-samsung-galaxy-a07-4g-128gb-4-gb?_lc=11</t>
-  </si>
-  <si>
     <t>/celular/celular-samsung-galaxy-s25-fe-5g-256gb-8-gb?_lc=11</t>
   </si>
   <si>
     <t>/celular/smartphone-samsung-galaxy-s24-ultra-5g-256gb-camera-quadrupla?_lc=11</t>
   </si>
   <si>
+    <t>/celular/celular-apple-iphone-16e-128gb-8-gb?_lc=11</t>
+  </si>
+  <si>
     <t>/celular/smartphone-apple-iphone-16-128gb-camera-dupla?_lc=11</t>
   </si>
   <si>
-    <t>/celular/celular-apple-iphone-16e-128gb-8-gb?_lc=11</t>
-  </si>
-  <si>
     <t>/celular/smartphone-apple-iphone-15-128gb-camera-dupla?_lc=11</t>
   </si>
   <si>
     <t>/celular/smartphone-samsung-galaxy-s24-5g-256gb?_lc=11</t>
   </si>
   <si>
+    <t>/celular/celular-motorola-moto-g86-5g-256gb-8-gb?_lc=11</t>
+  </si>
+  <si>
     <t>/celular/celular-samsung-galaxy-s25-plus-5g-256gb-12-gb?_lc=11</t>
   </si>
   <si>
-    <t>/celular/celular-motorola-moto-g86-5g-256gb-8-gb?_lc=11</t>
-  </si>
-  <si>
     <t>/celular/celular-samsung-galaxy-a07-4g-256gb-8-gb?_lc=11</t>
   </si>
   <si>
+    <t>/celular/celular-samsung-galaxy-s25-ultra-5g-256gb-12-gb?_lc=11</t>
+  </si>
+  <si>
     <t>/celular/celular-samsung-galaxy-s25-5g-256gb-12-gb?_lc=11</t>
   </si>
   <si>
-    <t>/celular/celular-samsung-galaxy-s25-ultra-5g-256gb-12-gb?_lc=11</t>
-  </si>
-  <si>
     <t>/celular/celular-samsung-a57-256gb-8-gb?_lc=11</t>
   </si>
   <si>
@@ -460,24 +460,24 @@
     <t>/celular/celular-samsung-galaxy-a36-5g-128gb-6-gb?_lc=11</t>
   </si>
   <si>
+    <t>/celular/celular-samsung-galaxy-s25-ultra-5g-512gb-12-gb?_lc=11</t>
+  </si>
+  <si>
+    <t>/celular/celular-xiaomi-x8-poco-pro-256gb-8-gb?_lc=11</t>
+  </si>
+  <si>
+    <t>/celular/celular-motorola-moto-edge-60-pro-5g-256gb-12-gb?_lc=11</t>
+  </si>
+  <si>
     <t>/celular/celular-xiaomi-redmi-15-256gb-8-gb?_lc=11</t>
   </si>
   <si>
-    <t>/celular/celular-motorola-moto-edge-60-pro-5g-256gb-12-gb?_lc=11</t>
-  </si>
-  <si>
-    <t>/celular/celular-xiaomi-x8-poco-pro-256gb-8-gb?_lc=11</t>
+    <t>/celular/celular-apple-iphone-17-pro-256gb?_lc=11</t>
   </si>
   <si>
     <t>/celular/smartphone-apple-iphone-15-pro-max-256gb-camera-tripla?_lc=11</t>
   </si>
   <si>
-    <t>/celular/celular-samsung-galaxy-s25-ultra-5g-512gb-12-gb?_lc=11</t>
-  </si>
-  <si>
-    <t>/celular/celular-apple-iphone-17-pro-256gb?_lc=11</t>
-  </si>
-  <si>
     <t>/celular/celular-samsung-galaxy-s26-ultra-5g-256gb?_lc=11</t>
   </si>
   <si>
@@ -487,16 +487,34 @@
     <t>/celular/smartphone-apple-iphone-16-256gb-camera-dupla?_lc=11</t>
   </si>
   <si>
+    <t>/celular/celular-samsung-galaxy-a26-256gb?_lc=11</t>
+  </si>
+  <si>
+    <t>/celular/celular-samsung-galaxy-s24-fe-5g-256gb-8-gb?_lc=11</t>
+  </si>
+  <si>
     <t>/celular/celular-samsung-galaxy-a25-5g-256gb-8-gb?_lc=11</t>
   </si>
   <si>
-    <t>/celular/celular-samsung-galaxy-a26-256gb?_lc=11</t>
+    <t>/celular/celular-motorola-edge-70-fusion-5g-256gb-8-gb?_lc=11</t>
+  </si>
+  <si>
+    <t>/celular/celular-samsung-a57-128gb-8-gb?_lc=11</t>
+  </si>
+  <si>
+    <t>/celular/celular-samsung-galaxy-a17-4g-128gb-4-gb?_lc=11</t>
   </si>
   <si>
     <t>/celular/celular-motorola-edge-60-fusion-5g-256gb-8-gb?_lc=11</t>
   </si>
   <si>
-    <t>/celular/celular-samsung-galaxy-s24-fe-5g-256gb-8-gb?_lc=11</t>
+    <t>/celular/smartphone-apple-iphone-14-plus-256gb-camera-dupla?_lc=11</t>
+  </si>
+  <si>
+    <t>/celular/celular-xiaomi-poco-c85-256gb-8-gb?_lc=11</t>
+  </si>
+  <si>
+    <t>/celular/celular-samsung-galaxy-a17-4g-256gb-8-gb?_lc=11</t>
   </si>
   <si>
     <t>/celular/smartphone-apple-iphone-13-256gb-ios?_lc=11</t>
@@ -505,39 +523,21 @@
     <t>/celular/celular-motorola-moto-g35-5g-128gb-12-gb?_lc=11</t>
   </si>
   <si>
-    <t>/celular/celular-samsung-a57-128gb-8-gb?_lc=11</t>
-  </si>
-  <si>
-    <t>/celular/celular-motorola-edge-70-fusion-5g-256gb-8-gb?_lc=11</t>
-  </si>
-  <si>
-    <t>/celular/celular-samsung-galaxy-a17-4g-128gb-4-gb?_lc=11</t>
-  </si>
-  <si>
-    <t>/celular/smartphone-apple-iphone-14-plus-256gb-camera-dupla?_lc=11</t>
-  </si>
-  <si>
-    <t>/celular/celular-xiaomi-poco-c85-256gb-8-gb?_lc=11</t>
-  </si>
-  <si>
-    <t>/celular/celular-samsung-galaxy-a17-4g-256gb-8-gb?_lc=11</t>
+    <t>/celular/celular-motorola-moto-g56-256gb-8-gb?_lc=11</t>
+  </si>
+  <si>
+    <t>/celular/celular-xiaomi-x8-poco-pro-512gb-12-gb?_lc=11</t>
   </si>
   <si>
     <t>/celular/celular-apple-iphone-17e-5g-256gb?_lc=11</t>
   </si>
   <si>
-    <t>/celular/celular-motorola-moto-g56-256gb-8-gb?_lc=11</t>
-  </si>
-  <si>
-    <t>/celular/celular-xiaomi-x8-poco-pro-512gb-12-gb?_lc=11</t>
+    <t>/celular/celular-motorola-moto-g-g06-128gb-4-gb?_lc=11</t>
   </si>
   <si>
     <t>/celular/celular-xiaomi-x8-poco-pro-max-512gb-12-gb?_lc=11</t>
   </si>
   <si>
-    <t>/celular/celular-motorola-moto-g-g06-128gb-4-gb?_lc=11</t>
-  </si>
-  <si>
     <t>/celular/celular-xiaomi-redmi-note-15-pro-5g-256gb-8-gb?_lc=11</t>
   </si>
   <si>
@@ -550,28 +550,28 @@
     <t>/celular/smartphone-apple-iphone-14-pro-256gb-camera-tripla?_lc=11</t>
   </si>
   <si>
+    <t>/celular/celular-motorola-edge-60-5g-512gb-12-gb?_lc=11</t>
+  </si>
+  <si>
     <t>/celular/celular-motorola-moto-g35-5g-256gb-12-gb?_lc=11</t>
   </si>
   <si>
-    <t>/celular/celular-motorola-edge-60-5g-512gb-12-gb?_lc=11</t>
-  </si>
-  <si>
     <t>/celular/smartphone-samsung-galaxy-a05s-128gb-camera-tripla?_lc=11</t>
   </si>
   <si>
+    <t>/celular/celular-apple-iphone-17-pro-max-512gb?_lc=11</t>
+  </si>
+  <si>
     <t>/celular/celular-motorola-moto-g75-5g-256gb-16-gb?_lc=11</t>
   </si>
   <si>
-    <t>/celular/celular-apple-iphone-17-pro-max-512gb?_lc=11</t>
-  </si>
-  <si>
-    <t>/celular/celular-motorola-edge-60-pro-512gb-12-gb?_lc=11</t>
+    <t>/celular/celular-xiaomi-redmi-note-14-pro-5g-256gb-8-gb?_lc=11</t>
   </si>
   <si>
     <t>/celular/celular-xiaomi-pocophone-poco-x7-pro-5g-256gb-8-gb?_lc=11</t>
   </si>
   <si>
-    <t>5578</t>
+    <t>5399</t>
   </si>
   <si>
     <t>2287</t>
@@ -586,45 +586,45 @@
     <t>2638</t>
   </si>
   <si>
-    <t>1374</t>
-  </si>
-  <si>
     <t>594</t>
   </si>
   <si>
+    <t>1405</t>
+  </si>
+  <si>
     <t>3123</t>
   </si>
   <si>
     <t>4249</t>
   </si>
   <si>
+    <t>3498</t>
+  </si>
+  <si>
     <t>4599</t>
   </si>
   <si>
-    <t>3498</t>
-  </si>
-  <si>
     <t>4099</t>
   </si>
   <si>
-    <t>2347</t>
+    <t>5579</t>
+  </si>
+  <si>
+    <t>1494</t>
   </si>
   <si>
     <t>4047</t>
   </si>
   <si>
-    <t>1494</t>
-  </si>
-  <si>
     <t>789</t>
   </si>
   <si>
+    <t>5199</t>
+  </si>
+  <si>
     <t>3758</t>
   </si>
   <si>
-    <t>5199</t>
-  </si>
-  <si>
     <t>2443</t>
   </si>
   <si>
@@ -640,43 +640,61 @@
     <t>1399</t>
   </si>
   <si>
+    <t>5865</t>
+  </si>
+  <si>
+    <t>2199</t>
+  </si>
+  <si>
+    <t>2591</t>
+  </si>
+  <si>
     <t>1175</t>
   </si>
   <si>
-    <t>2591</t>
-  </si>
-  <si>
-    <t>2199</t>
+    <t>7892</t>
   </si>
   <si>
     <t>5642</t>
   </si>
   <si>
-    <t>5865</t>
-  </si>
-  <si>
-    <t>7892</t>
-  </si>
-  <si>
     <t>6652</t>
   </si>
   <si>
     <t>1699</t>
   </si>
   <si>
-    <t>5399</t>
+    <t>4859</t>
+  </si>
+  <si>
+    <t>1359</t>
+  </si>
+  <si>
+    <t>2775</t>
   </si>
   <si>
     <t>1131</t>
   </si>
   <si>
-    <t>1421</t>
-  </si>
-  <si>
-    <t>1715</t>
-  </si>
-  <si>
-    <t>2775</t>
+    <t>2198</t>
+  </si>
+  <si>
+    <t>1954</t>
+  </si>
+  <si>
+    <t>729</t>
+  </si>
+  <si>
+    <t>1753</t>
+  </si>
+  <si>
+    <t>3500</t>
+  </si>
+  <si>
+    <t>939</t>
+  </si>
+  <si>
+    <t>1164</t>
   </si>
   <si>
     <t>3009</t>
@@ -685,39 +703,18 @@
     <t>917</t>
   </si>
   <si>
-    <t>1954</t>
-  </si>
-  <si>
-    <t>1847</t>
-  </si>
-  <si>
-    <t>729</t>
-  </si>
-  <si>
-    <t>3325</t>
-  </si>
-  <si>
-    <t>939</t>
-  </si>
-  <si>
-    <t>1164</t>
+    <t>2649</t>
   </si>
   <si>
     <t>4499</t>
   </si>
   <si>
-    <t>1359</t>
-  </si>
-  <si>
-    <t>2649</t>
+    <t>598</t>
   </si>
   <si>
     <t>3499</t>
   </si>
   <si>
-    <t>598</t>
-  </si>
-  <si>
     <t>1919</t>
   </si>
   <si>
@@ -730,22 +727,22 @@
     <t>4084</t>
   </si>
   <si>
+    <t>2124</t>
+  </si>
+  <si>
     <t>999</t>
   </si>
   <si>
-    <t>2124</t>
-  </si>
-  <si>
     <t>635</t>
   </si>
   <si>
+    <t>10169</t>
+  </si>
+  <si>
     <t>1785</t>
   </si>
   <si>
-    <t>10169</t>
-  </si>
-  <si>
-    <t>2999</t>
+    <t>1828</t>
   </si>
   <si>
     <t>2100</t>
@@ -766,45 +763,45 @@
     <t>https://i.zst.com.br/thumbs/45/39/14/-1591251808.jpg</t>
   </si>
   <si>
+    <t>https://i.zst.com.br/thumbs/45/f/35/-1597645208.jpg</t>
+  </si>
+  <si>
     <t>https://i.zst.com.br/thumbs/45/16/30/-1584401187.jpg</t>
   </si>
   <si>
-    <t>https://i.zst.com.br/thumbs/45/f/35/-1597645208.jpg</t>
-  </si>
-  <si>
     <t>https://i.zst.com.br/thumbs/45/30/14/-1591252595.jpg</t>
   </si>
   <si>
     <t>https://i.zst.com.br/thumbs/45/30/17/-1202498267.jpg</t>
   </si>
   <si>
+    <t>https://i.zst.com.br/thumbs/45/12/32/-1472883387.jpg</t>
+  </si>
+  <si>
     <t>https://i.zst.com.br/thumbs/45/16/f/-1346812222.jpg</t>
   </si>
   <si>
-    <t>https://i.zst.com.br/thumbs/45/12/32/-1472883387.jpg</t>
-  </si>
-  <si>
     <t>https://i.zst.com.br/thumbs/45/19/31/-1113972290.jpg</t>
   </si>
   <si>
     <t>https://i.zst.com.br/thumbs/45/3d/11/-1202542340.jpg</t>
   </si>
   <si>
+    <t>https://i.zst.com.br/thumbs/45/2e/2d/-1603821631.jpg</t>
+  </si>
+  <si>
     <t>https://i.zst.com.br/thumbs/45/37/2f/-1451536322.jpg</t>
   </si>
   <si>
-    <t>https://i.zst.com.br/thumbs/45/2e/2d/-1603821631.jpg</t>
-  </si>
-  <si>
     <t>https://i.zst.com.br/thumbs/45/2c/35/-1597643414.jpg</t>
   </si>
   <si>
+    <t>https://i.zst.com.br/thumbs/45/18/3d/-1449484750.jpg</t>
+  </si>
+  <si>
     <t>https://i.zst.com.br/thumbs/45/37/3b/-1449465281.jpg</t>
   </si>
   <si>
-    <t>https://i.zst.com.br/thumbs/45/18/3d/-1449484750.jpg</t>
-  </si>
-  <si>
     <t>https://i.zst.com.br/thumbs/45/24/14/-1693348668.jpg</t>
   </si>
   <si>
@@ -820,24 +817,24 @@
     <t>https://i.zst.com.br/thumbs/45/11/f/-1524507737.jpg</t>
   </si>
   <si>
+    <t>https://i.zst.com.br/thumbs/45/1c/14/-1449500134.jpg</t>
+  </si>
+  <si>
+    <t>https://i.zst.com.br/thumbs/45/2/12/-1683989765.jpg</t>
+  </si>
+  <si>
+    <t>https://i.zst.com.br/thumbs/45/1a/1c/-1529478118.jpg</t>
+  </si>
+  <si>
     <t>https://i.zst.com.br/thumbs/45/3a/3a/-1598683126.jpg</t>
   </si>
   <si>
-    <t>https://i.zst.com.br/thumbs/45/1a/1c/-1529478118.jpg</t>
-  </si>
-  <si>
-    <t>https://i.zst.com.br/thumbs/45/2/12/-1683989765.jpg</t>
+    <t>https://i.zst.com.br/thumbs/45/3f/1b/-1584074872.jpg</t>
   </si>
   <si>
     <t>https://i.zst.com.br/thumbs/45/a/13/-1114650735.jpg</t>
   </si>
   <si>
-    <t>https://i.zst.com.br/thumbs/45/1c/14/-1449500134.jpg</t>
-  </si>
-  <si>
-    <t>https://i.zst.com.br/thumbs/45/3f/1b/-1584074872.jpg</t>
-  </si>
-  <si>
     <t>https://i.zst.com.br/thumbs/45/2a/1b/-1678471943.jpg</t>
   </si>
   <si>
@@ -847,16 +844,34 @@
     <t>https://i.zst.com.br/thumbs/45/1c/37/-1347442557.jpg</t>
   </si>
   <si>
+    <t>https://i.zst.com.br/thumbs/45/30/33/-1475648263.jpg</t>
+  </si>
+  <si>
+    <t>https://i.zst.com.br/thumbs/45/5/15/-1358966033.jpg</t>
+  </si>
+  <si>
     <t>https://i.zst.com.br/thumbs/45/29/33/-1421244724.jpg</t>
   </si>
   <si>
-    <t>https://i.zst.com.br/thumbs/45/30/33/-1475648263.jpg</t>
+    <t>https://i.zst.com.br/thumbs/45/d/15/-1680059930.jpg</t>
+  </si>
+  <si>
+    <t>https://i.zst.com.br/thumbs/45/15/14/-1693349843.jpg</t>
+  </si>
+  <si>
+    <t>https://i.zst.com.br/thumbs/45/39/30/-1678916430.jpg</t>
   </si>
   <si>
     <t>https://i.zst.com.br/thumbs/45/d/13/-1500036474.jpg</t>
   </si>
   <si>
-    <t>https://i.zst.com.br/thumbs/45/5/15/-1358966033.jpg</t>
+    <t>https://i.zst.com.br/thumbs/45/31/1c/-871936652.jpg</t>
+  </si>
+  <si>
+    <t>https://i.zst.com.br/thumbs/45/14/37/-1591284000.jpg</t>
+  </si>
+  <si>
+    <t>https://i.zst.com.br/thumbs/45/35/30/-1678917590.jpg</t>
   </si>
   <si>
     <t>https://i.zst.com.br/thumbs/45/23/11/-747056146.jpg</t>
@@ -865,39 +880,21 @@
     <t>https://i.zst.com.br/thumbs/45/29/2e/-1554937995.jpg</t>
   </si>
   <si>
-    <t>https://i.zst.com.br/thumbs/45/15/14/-1693349843.jpg</t>
-  </si>
-  <si>
-    <t>https://i.zst.com.br/thumbs/45/d/15/-1680059930.jpg</t>
-  </si>
-  <si>
-    <t>https://i.zst.com.br/thumbs/45/39/30/-1678916430.jpg</t>
-  </si>
-  <si>
-    <t>https://i.zst.com.br/thumbs/45/31/1c/-871936652.jpg</t>
-  </si>
-  <si>
-    <t>https://i.zst.com.br/thumbs/45/14/37/-1591284000.jpg</t>
-  </si>
-  <si>
-    <t>https://i.zst.com.br/thumbs/45/35/30/-1678917590.jpg</t>
+    <t>https://i.zst.com.br/thumbs/45/10/30/-1532643273.jpg</t>
+  </si>
+  <si>
+    <t>https://i.zst.com.br/thumbs/45/3e/33/-1683990601.jpg</t>
   </si>
   <si>
     <t>https://i.zst.com.br/thumbs/45/11/12/-1679706169.jpg</t>
   </si>
   <si>
-    <t>https://i.zst.com.br/thumbs/45/10/30/-1532643273.jpg</t>
-  </si>
-  <si>
-    <t>https://i.zst.com.br/thumbs/45/3e/33/-1683990601.jpg</t>
+    <t>https://i.zst.com.br/thumbs/45/11/11/-1590231539.jpg</t>
   </si>
   <si>
     <t>https://i.zst.com.br/thumbs/45/d/33/-1683996479.jpg</t>
   </si>
   <si>
-    <t>https://i.zst.com.br/thumbs/45/11/11/-1590231539.jpg</t>
-  </si>
-  <si>
     <t>https://i.zst.com.br/thumbs/45/2b/3f/-1687085680.jpg</t>
   </si>
   <si>
@@ -910,22 +907,22 @@
     <t>https://i.zst.com.br/thumbs/45/12/11/-845276527.jpg</t>
   </si>
   <si>
+    <t>https://i.zst.com.br/thumbs/45/3a/1a/-1505387439.jpg</t>
+  </si>
+  <si>
     <t>https://i.zst.com.br/thumbs/45/b/14/-1533234478.jpg</t>
   </si>
   <si>
-    <t>https://i.zst.com.br/thumbs/45/3a/1a/-1505387439.jpg</t>
-  </si>
-  <si>
     <t>https://i.zst.com.br/thumbs/45/3f/15/-1206545191.jpg</t>
   </si>
   <si>
+    <t>https://i.zst.com.br/thumbs/45/3/1b/-1584070252.jpg</t>
+  </si>
+  <si>
     <t>https://i.zst.com.br/thumbs/45/1e/36/-1420399903.jpg</t>
   </si>
   <si>
-    <t>https://i.zst.com.br/thumbs/45/3/1b/-1584070252.jpg</t>
-  </si>
-  <si>
-    <t>https://i.zst.com.br/thumbs/45/2a/33/-1505424683.jpg</t>
+    <t>https://i.zst.com.br/thumbs/45/2e/16/-1459965948.jpg</t>
   </si>
   <si>
     <t>https://i.zst.com.br/thumbs/45/6/f/-1532413784.jpg</t>
@@ -1333,7 +1330,7 @@
         <v>185</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -1350,7 +1347,7 @@
         <v>186</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -1367,7 +1364,7 @@
         <v>187</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -1384,7 +1381,7 @@
         <v>188</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -1401,7 +1398,7 @@
         <v>189</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -1418,7 +1415,7 @@
         <v>190</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -1435,7 +1432,7 @@
         <v>191</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -1452,7 +1449,7 @@
         <v>192</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -1469,7 +1466,7 @@
         <v>193</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -1486,7 +1483,7 @@
         <v>194</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -1503,7 +1500,7 @@
         <v>195</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -1520,7 +1517,7 @@
         <v>196</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="14" spans="1:5">
@@ -1537,7 +1534,7 @@
         <v>197</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="15" spans="1:5">
@@ -1554,7 +1551,7 @@
         <v>198</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="16" spans="1:5">
@@ -1571,7 +1568,7 @@
         <v>199</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -1588,7 +1585,7 @@
         <v>200</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="18" spans="1:5">
@@ -1605,7 +1602,7 @@
         <v>201</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="19" spans="1:5">
@@ -1622,7 +1619,7 @@
         <v>202</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="20" spans="1:5">
@@ -1639,7 +1636,7 @@
         <v>203</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="21" spans="1:5">
@@ -1656,7 +1653,7 @@
         <v>204</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="22" spans="1:5">
@@ -1673,7 +1670,7 @@
         <v>205</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="23" spans="1:5">
@@ -1690,7 +1687,7 @@
         <v>206</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="24" spans="1:5">
@@ -1707,7 +1704,7 @@
         <v>207</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -1724,7 +1721,7 @@
         <v>208</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
     </row>
     <row r="26" spans="1:5">
@@ -1741,7 +1738,7 @@
         <v>209</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="27" spans="1:5">
@@ -1758,7 +1755,7 @@
         <v>210</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="28" spans="1:5">
@@ -1775,7 +1772,7 @@
         <v>211</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="29" spans="1:5">
@@ -1792,7 +1789,7 @@
         <v>212</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="30" spans="1:5">
@@ -1809,7 +1806,7 @@
         <v>213</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="31" spans="1:5">
@@ -1826,7 +1823,7 @@
         <v>214</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="32" spans="1:5">
@@ -1843,7 +1840,7 @@
         <v>215</v>
       </c>
       <c r="E32" s="2" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="33" spans="1:5">
@@ -1860,7 +1857,7 @@
         <v>216</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="34" spans="1:5">
@@ -1877,7 +1874,7 @@
         <v>217</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="35" spans="1:5">
@@ -1894,7 +1891,7 @@
         <v>218</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="36" spans="1:5">
@@ -1911,7 +1908,7 @@
         <v>219</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="37" spans="1:5">
@@ -1928,7 +1925,7 @@
         <v>220</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="38" spans="1:5">
@@ -1945,7 +1942,7 @@
         <v>221</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="39" spans="1:5">
@@ -1962,7 +1959,7 @@
         <v>222</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="40" spans="1:5">
@@ -1979,7 +1976,7 @@
         <v>223</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="41" spans="1:5">
@@ -1996,7 +1993,7 @@
         <v>224</v>
       </c>
       <c r="E41" s="2" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="42" spans="1:5">
@@ -2013,7 +2010,7 @@
         <v>225</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="43" spans="1:5">
@@ -2030,7 +2027,7 @@
         <v>226</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="44" spans="1:5">
@@ -2047,7 +2044,7 @@
         <v>227</v>
       </c>
       <c r="E44" s="2" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="45" spans="1:5">
@@ -2064,7 +2061,7 @@
         <v>228</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="46" spans="1:5">
@@ -2078,10 +2075,10 @@
         <v>169</v>
       </c>
       <c r="D46" t="s">
-        <v>229</v>
+        <v>217</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="47" spans="1:5">
@@ -2095,10 +2092,10 @@
         <v>170</v>
       </c>
       <c r="D47" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="E47" s="2" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
     </row>
     <row r="48" spans="1:5">
@@ -2112,10 +2109,10 @@
         <v>171</v>
       </c>
       <c r="D48" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
     </row>
     <row r="49" spans="1:5">
@@ -2129,10 +2126,10 @@
         <v>172</v>
       </c>
       <c r="D49" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="50" spans="1:5">
@@ -2146,10 +2143,10 @@
         <v>173</v>
       </c>
       <c r="D50" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="E50" s="2" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="51" spans="1:5">
@@ -2163,10 +2160,10 @@
         <v>174</v>
       </c>
       <c r="D51" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
     </row>
     <row r="52" spans="1:5">
@@ -2180,10 +2177,10 @@
         <v>175</v>
       </c>
       <c r="D52" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="53" spans="1:5">
@@ -2197,10 +2194,10 @@
         <v>176</v>
       </c>
       <c r="D53" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="54" spans="1:5">
@@ -2214,10 +2211,10 @@
         <v>177</v>
       </c>
       <c r="D54" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="55" spans="1:5">
@@ -2231,10 +2228,10 @@
         <v>178</v>
       </c>
       <c r="D55" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
     </row>
     <row r="56" spans="1:5">
@@ -2248,10 +2245,10 @@
         <v>179</v>
       </c>
       <c r="D56" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="E56" s="2" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="57" spans="1:5">
@@ -2265,10 +2262,10 @@
         <v>180</v>
       </c>
       <c r="D57" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="58" spans="1:5">
@@ -2282,10 +2279,10 @@
         <v>181</v>
       </c>
       <c r="D58" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
     </row>
     <row r="59" spans="1:5">
@@ -2299,10 +2296,10 @@
         <v>182</v>
       </c>
       <c r="D59" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="E59" s="2" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
     </row>
     <row r="60" spans="1:5">
@@ -2316,10 +2313,10 @@
         <v>183</v>
       </c>
       <c r="D60" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="E60" s="2" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="61" spans="1:5">
@@ -2333,10 +2330,10 @@
         <v>184</v>
       </c>
       <c r="D61" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="E61" s="2" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
   </sheetData>

</xml_diff>